<commit_message>
try to multiple round fix
</commit_message>
<xml_diff>
--- a/data/addition.xlsx
+++ b/data/addition.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,150 +459,72 @@
           <t>差异</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>difflib</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@performance/hp-arkui-use-transition-to-replace-animateto</t>
+          <t>@performance/high-frequency-log-check</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Use transition for component transition animation</t>
+          <t>不建议在高频函数中使用Hilog或者其它打印日志的方式。</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>@Entry
+          <t>import hilog from '@ohos.hilog';
+@Entry
 @Component
-struct MyComponent {
-  @State mOpacity: number = 1;
-  @State show: boolean = true;
+struct App {
   build() {
-    Column() {
-      Row() {
-        if (this.show) {
-          Text('value')
-            .opacity(this.mOpacity)
-        }
-      }
+    Canvas(()=&gt;{})
       .width('100%')
-      .height(100)
-      .justifyContent(FlexAlign.Center)
-      Text('toggle state')
-        .onClick(() =&gt; {
-          this.show = true;
-          animateTo({
-            duration: 1000, onFinish: () =&gt; {
-              if (this.mOpacity === 0) {
-                this.show = false;
-              }
-            }
-          }, () =&gt; {
-            this.mOpacity = this.mOpacity === 1 ? 0 : 1;
-          })
-        })
-    }
+      .height('100%')
+      .onScroll((xOffset: number, yOffset: number) =&gt; {
+        console.info(1001, 'App', 'onScroll')
+    })
   }
 }</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>原来的代码中使用了animtaeTo函数，通过改变opacity来使得点击后Text('value')慢慢消失，这会造成帧率的丢失，建议使用.trainsition的属性来进行改变</t>
+          <t>onScroll 是高频事件之一。在布局中，每次滚动都会触发这个函数。如果在该函数中使用 console.info 进行日志记录，可能导致性能问题。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>@Entry
+          <t>import hilog from '@ohos.hilog';
+@Entry
 @Component
-struct MyComponent {
-  @State show: boolean = true;
+struct App {
   build() {
-    Column() {
-      Row() {
-        if (this.show) {
-          Text('value')// Set id to make transition interruptible
-            .id('myText')
-            .transition(TransitionEffect.OPACITY.animation({ duration: 1000 }))
-        }
-      }.width('100%')
-      .height(100)
-      .justifyContent(FlexAlign.Center)
-      Text('toggle state')
-        .onClick(() =&gt; {
-          // Through transition, animates the appearance or disappearance of transparency.
-          this.show = !this.show;
-        })
-    }
+    Canvas(()=&gt;{})
+      .width('100%')
+      .height('100%')
+      .onScroll((xOffset: number, yOffset: number) =&gt; {
+        const TAG = 'onScroll'
+    })
   }
 }</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>在修复代码样例中，相比于问题代码样例，有以下几个明显的差异：
-1. **去除不再使用的状态**:
-   - 修复代码中去除了 `mOpacity` 的状态，只保留了 `show` 状态。这样简化了状态管理，不需要手动管理不透明度。
-2. **添加 ID 属性**:
-   - 修复代码样例在 `Text('value')` 上添加了 `.id('myText')`，这是为了使得过渡动画可中断，增强了动画的控制性。
-3. **使用过渡效果**:
-   - 修复代码中对 `Text('value')` 添加了 `.transition(TransitionEffect.OPACITY.animation({ duration: 1000 }))`，使用了过渡效果来处理透明度的变化。相较于问题代码中使用 `animateTo` 进行手动动画，修复代码通过使用过渡效果可以更简洁地实现动画。
-4. **简化点击处理**:
-   - 在修复代码中，点击事件直接切换 `show` 状态（`this.show = !this.show;`），而不是先将 `this.show` 设置为 `true`，然后通过 `animateTo` 更新不透明度。这种写法简化了切换逻辑。
-5. **去掉动画结束后的状态检查**:
-   - 修复代码没有进行动画完成后的状态检查（`if (this.mOpacity === 0) { this.show = false; }`），取而代之的是直接通过过渡效果来处理显示和隐藏。
-通过上述差异，修复后的代码实现了更简洁和有效的动画表现，同时也避免了潜在的逻辑复杂性。</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  @Entry
-  @Component
-  struct MyComponent {
--   @State mOpacity: number = 1;
-    @State show: boolean = true;
-    build() {
-      Column() {
-        Row() {
-          if (this.show) {
--           Text('value')
--             .opacity(this.mOpacity)
-+           Text('value')// Set id to make transition interruptible
-+             .id('myText')
-+             .transition(TransitionEffect.OPACITY.animation({ duration: 1000 }))
-          }
--       }
--       .width('100%')
-+       }.width('100%')
-?       +
-        .height(100)
-        .justifyContent(FlexAlign.Center)
-        Text('toggle state')
-          .onClick(() =&gt; {
-+           // Through transition, animates the appearance or disappearance of transparency.
--           this.show = true;
-?                        ^^^
-+           this.show = !this.show;
-?                       + ^^^^^^^^
--           animateTo({
--             duration: 1000, onFinish: () =&gt; {
--               if (this.mOpacity === 0) {
--                 this.show = false;
--               }
--             }
--           }, () =&gt; {
--             this.mOpacity = this.mOpacity === 1 ? 0 : 1;
--           })
-          })
-      }
-    }
-  }</t>
+          <t>在提供的两个代码样例中，修复代码相对于问题代码的主要差异如下：
+1. **日志输出的更改**：
+   - 在问题代码样例中，`onScroll` 方法内部有一行日志输出代码：
+     ```javascript
+     console.info(1001, 'App', 'onScroll')
+     ```
+     这个语句将输出一些调试信息。它显示了一个标识符（1001）、组件名（'App'）和一个消息（'onScroll'）。
+   - 在修复代码样例中，`onScroll` 方法内部去除了日志输出语句，仅仅保留了一个常量定义：
+     ```javascript
+     const TAG = 'onScroll'
+     ```
+     这表示修复代码没有记录日志信息，而是定义了一个常量。
+总结来说，修复代码的主要差异是去掉了原有的日志输出，改为定义了常量 `TAG`，这可能表明修复的目的是避免过多的日志输出，或者将来准备使用该常量，但修复代码没有提供对 `TAG` 的实际使用。</t>
         </is>
       </c>
     </row>

</xml_diff>